<commit_message>
Commit map and config updates
</commit_message>
<xml_diff>
--- a/docs/design/蛋仔--大富翁--地图示例.xlsx
+++ b/docs/design/蛋仔--大富翁--地图示例.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\eggitor\1_开发中\大富翁\monopoly\design\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\eggitor\1_开发中\大富翁\策划案\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B22C39F5-1A73-476A-BCDA-86933EB77B38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4215E74A-DD01-455F-9E2C-1D6C16F1793E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="地图示例" sheetId="1" r:id="rId1"/>
@@ -448,25 +448,28 @@
     <t>税务局38</t>
   </si>
   <si>
-    <t>机会卡41</t>
-  </si>
-  <si>
-    <t>机会卡42</t>
-  </si>
-  <si>
     <t>机会卡43</t>
   </si>
   <si>
     <t>道具卡44</t>
   </si>
   <si>
-    <t>道具卡45</t>
-  </si>
-  <si>
     <t>机会卡40</t>
   </si>
   <si>
     <t>黑市39</t>
+  </si>
+  <si>
+    <t>道具卡41</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>道具卡42</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>机会卡45</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -689,7 +692,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -734,9 +737,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1413,8 +1413,8 @@
       <c r="E13" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="F13" s="28" t="s">
-        <v>115</v>
+      <c r="F13" s="6" t="s">
+        <v>119</v>
       </c>
       <c r="G13" s="3" t="s">
         <v>92</v>
@@ -1422,7 +1422,7 @@
       <c r="H13" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="I13" s="29" t="s">
+      <c r="I13" s="28" t="s">
         <v>94</v>
       </c>
       <c r="J13" s="7" t="s">
@@ -1441,13 +1441,13 @@
       </c>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
-      <c r="F14" s="29" t="s">
+      <c r="F14" s="28" t="s">
         <v>106</v>
       </c>
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
-      <c r="J14" s="29" t="s">
+      <c r="J14" s="28" t="s">
         <v>95</v>
       </c>
       <c r="M14" s="9" t="s">
@@ -1503,7 +1503,7 @@
         <v>5</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>101</v>
@@ -1515,10 +1515,10 @@
         <v>103</v>
       </c>
       <c r="F17" s="10" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="H17" s="3" t="s">
         <v>109</v>
@@ -1527,7 +1527,7 @@
         <v>110</v>
       </c>
       <c r="J17" s="5" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="M17" s="9" t="s">
         <v>64</v>
@@ -1556,7 +1556,7 @@
       <c r="A19">
         <v>7</v>
       </c>
-      <c r="B19" s="29" t="s">
+      <c r="B19" s="28" t="s">
         <v>84</v>
       </c>
       <c r="C19" s="2"/>
@@ -1567,7 +1567,7 @@
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
       <c r="I19" s="2"/>
-      <c r="J19" s="29" t="s">
+      <c r="J19" s="28" t="s">
         <v>99</v>
       </c>
       <c r="M19" s="9" t="s">
@@ -1578,11 +1578,11 @@
       <c r="A20">
         <v>8</v>
       </c>
-      <c r="B20" s="29" t="s">
+      <c r="B20" s="28" t="s">
         <v>83</v>
       </c>
-      <c r="F20" s="6" t="s">
-        <v>119</v>
+      <c r="F20" s="5" t="s">
+        <v>121</v>
       </c>
       <c r="J20" s="4" t="s">
         <v>100</v>
@@ -1604,8 +1604,8 @@
       <c r="E21" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="F21" s="5" t="s">
-        <v>116</v>
+      <c r="F21" s="6" t="s">
+        <v>120</v>
       </c>
       <c r="G21" s="3" t="s">
         <v>69</v>

</xml_diff>